<commit_message>
Svetainė v2: EN/LT, ataskaitos su išnašomis, ESG pagal šabloną, ISIN sąrašo puslapis
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZCssjCF43KM8LCnCdqfwt
</commit_message>
<xml_diff>
--- a/docs/files/ignitis/ignitis_6M2026_lt.xlsx
+++ b/docs/files/ignitis/ignitis_6M2026_lt.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +473,11 @@
           <t>6M2026</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Šaltiniai</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -492,6 +498,11 @@
       <c r="F2" s="2" t="n">
         <v>1497.5</v>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.23</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -516,6 +527,11 @@
       <c r="F3" s="2" t="n">
         <v>306.6</v>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.11; S1 p.5; S4 p.14; S5</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -540,6 +556,11 @@
       <c r="F4" s="2" t="n">
         <v>303.5</v>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.11; S4 p.14</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -564,6 +585,11 @@
       <c r="F5" s="2" t="n">
         <v>115.8</v>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.11; S4 p.14; S5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -588,6 +614,11 @@
       <c r="F6" s="2" t="n">
         <v>113.2</v>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.23; S4 p.14</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -611,6 +642,11 @@
       </c>
       <c r="F7" s="2" t="n">
         <v>306.1</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.11; S1 p.5; S4 p.14; S5</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -632,6 +668,11 @@
       <c r="F8" s="2" t="n">
         <v>251.4</v>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.29</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -652,6 +693,11 @@
       <c r="F9" s="2" t="n">
         <v>5.3</v>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.29</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -674,6 +720,11 @@
       <c r="F10" s="2" t="n">
         <v>1925.3</v>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.10; S4 p.14</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -696,6 +747,11 @@
       <c r="F11" s="2" t="n">
         <v>3.49</v>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.10; S4 p.14</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -718,6 +774,11 @@
       <c r="F12" s="2" t="n">
         <v>22.2</v>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.10; S4 p.14</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -739,6 +800,11 @@
       </c>
       <c r="F13" s="2" t="n">
         <v>6.7</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.11; S4 p.14</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -760,6 +826,11 @@
       <c r="F14" s="2" t="n">
         <v>2636.1</v>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.33</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -780,6 +851,11 @@
       <c r="F15" s="2" t="n">
         <v>6339.2</v>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.33</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -802,6 +878,11 @@
       <c r="F16" s="2" t="n">
         <v>0.704</v>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>S2; S4; S5</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -823,6 +904,11 @@
       </c>
       <c r="F17" s="2" t="n">
         <v>2.1</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>S1 p.11; S5</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1322,198 +1408,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Klausimas</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Būsena</t>
+          <t>Question</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Įrodymas</t>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Anglies (kasyba ar anglies elektrinės) dalis pajamose mažesnė nei 5 %</t>
+          <t>Exclusionary screening (companies)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>☑ Atitinka</t>
+          <t>Yes, the company is not involved in excluded sectors: controversial and nuclear weapons, tobacco, gambling and restricted sectors in fossil fuel</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Anglies generacijos nėra; 2025 m. ataskaitoje anglis minima tik rinkos kontekste [S4].</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ginklų, tabako ir lošimų veiklos nėra. Anglies generacijos nėra, naftos ir dujų žvalgybos nėra [S4]. Turi dujomis kūrenamą Elektrėnų kompleksą (rezervinė galia) ir tiekia dujas klientams – SEB iškastinio kuro politika tokios veiklos nedraudžia (ribojama anglis &gt;5 % pajamų ir nauja žvalgyba).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Nėra naujos naftos ir dujų žvalgybos / netradicinės naftos</t>
+          <t>Exclusionary screening (companies)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>☑ Atitinka</t>
+          <t>Yes, the company does not have red flag/signal related to controversies based on UN Global Compact, OECD Guidelines for Multinational Enterprises or any other relevant principles/standards</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Naftos ir dujų žvalgybos nėra. Turi dujomis kūrenamą Elektrėnų kompleksą (rezervinė galia) ir parduoda dujas klientams; dėl didesnės dujų generacijos žalioji generacijos dalis sumažėjo iki 70,2 % [S4].</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Raudonų signalų (UNGC, OECD pažeidimų) viešuose šaltiniuose ir naujienų paieškoje nerasta (2026-10-22). Ignitis skelbia, kad laikosi UN Global Compact principų [S4].</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Nėra sąsajų su kontroversiškais ginklais, tabaku ar lošimais</t>
+          <t>Exclusionary screening (companies)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>☑ Atitinka</t>
+          <t>Yes, the company is not in the list of sanctions (add a screenshot)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Veiklos segmentuose tokios veiklos nėra [S1].</t>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tikrina analitikas vidinėmis priemonėmis (pridėti ekrano nuotrauką).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Nėra rimtų neišspręstų skandalų (korupcija, žmogaus teisės, aplinka)</t>
+          <t>Exclusionary screening (companies)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>☐ Reikia peržiūrėti</t>
+          <t>Yes, issues were not identified from adverse media checks (add a screenshot)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Didelių neišspręstų skandalų greitoje paieškoje (2026-10-22) nerasta. 2026 m. vasarį – mirtinas nelaimingas atsitikimas su rangovo darbuotoju [S10].</t>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Automatinė naujienų paieška (LT, LV, EE, EN; 30 d.) neigiamų antraščių nerado. Analitikas patvirtina ir prideda ekrano nuotrauką.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Emisijų mažinimo tikslai (Paryžiaus / SBTi) ir pereinamojo laikotarpio planas</t>
+          <t>ESG integration and positive screening (positive answers imply higher allocation)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>☑ Atitinka</t>
+          <t>Yes, the company is promoting environmental or social characteristics (activities, ESG policy, good ESG rating, etc)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>SBTi patvirtino trumpojo ir ilgojo laikotarpio tikslus pagal 1,5 °C trajektoriją; nulinė emisija iki 2050 m. ar anksčiau [S4 p.10].</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pagrindinė veikla – žalioji generacija (įrengta 2,1 GW, statoma 0,6 GW) ir elektros tinklai [S1 p.11]; žaliosios obligacijos ir nauja ES žaliųjų obligacijų standarto (EuGB) obligacija [S9].</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tvarumo ataskaitos (CSRD/ESRS ar GRI), atskleistos 1–3 apimties emisijos</t>
+          <t>ESG integration and positive screening (positive answers imply higher allocation)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>☑ Atitinka</t>
+          <t>Yes, the activities of the company or it’s strategy is aligned with the taxonomy and/or Paris agreement targets (e.g. net zero commitment)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Integruota metinė ataskaita su ŠESD duomenimis: bendros emisijos 4,49 mln. t CO2e (+10,1 %), 1 apimtis +54,7 %; anglies intensyvumas (1+2) I ketv. 214 g/kWh [S4; S10].</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ES taksonomiją atitinkančios investicijos 2025 m. – 84,7 % [S4]. SBTi patvirtino tikslus pagal 1,5 °C trajektoriją; nulinė emisija iki 2050 m. ar anksčiau [S4 p.10].</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Teigiamas indėlis (žaliosios pajamos / investicijos, ES taksonomija, žaliosios obligacijos)</t>
+          <t>ESG integration and positive screening (positive answers imply higher allocation)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>☑ Atitinka</t>
+          <t>Yes, the company does not have yellow flag/signal related to controversies based on UN Global Compact or any other relevant principles/standards</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ES taksonomiją atitinkančios investicijos 2025 m. – 84,7 %; žaliosios obligacijos ir nauja EuGB obligacija [S4; S9].</t>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Galimas geltonas signalas: 2026 m. vasarį žuvo rangovo darbuotojas [S10]. 1 apimties emisijos 2025 m. išaugo 54,7 % dėl didesnės dujų generacijos [S4].</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Valdysena – nepriklausoma valdyba, antikorupcijos ir pranešėjų politikos</t>
+          <t>ESG integration and positive screening (positive answers imply higher allocation)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>☐ Reikia peržiūrėti</t>
+          <t>Yes, the company fulfills the expectations from SEB thematic and sector policies</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Valstybės valdoma (~75 %), listinguojama Nasdaq Vilnius ir LSE. Valdybos nepriklausomumas automatiškai netikrintas.</t>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Iškastinio kuro politika – atitinka (anglies ir naftos / dujų žvalgybos nėra). Elektros ir atsinaujinančios energijos, klimato ir žmogaus teisių politikų turinys automatiškai neperskaitytas (SEB PDF blokuoja automatinį skaitymą) – reikia rankinės patikros.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Socialiniai aspektai – sauga, darbo ir žmogaus teisių politikos</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>☐ Reikia peržiūrėti</t>
+          <t>Is there a need for pro-active engagement with the company?</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Sveikatos ir saugos rizika: mirtinas atvejis 2026 m. vasarį [S10]. Žmogaus teisių politika automatiškai netikrinta.</t>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Būtinybės nenustatyta. Galimos temos: dujų generacijos dalis ir 1 apimties emisijų augimas, rangovų sauga.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Klausimai įsitraukimui su emitentu</t>
+          <t>Indicators</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>☐ Reikia peržiūrėti</t>
+          <t>Yes, the indicators of the company support the targets of sustainability and PAI indicators followed by the Fund</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Siūlomi klausimai: 1 apimties emisijų augimas dėl dujų generacijos; rangovų sauga; FFO / skolos grįžimas į ≥23 %.</t>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Turimi PAI duomenys: bendros ŠESD emisijos 4,49 mln. t CO2e (+10,1 %) [S4]; anglies intensyvumas (1+2) 214 g CO2e/kWh I ketv. 2026 (−12,8 %) [S10]; taksonomiją atitinkančios investicijos 84,7 % [S4]. Palyginti su fondo tikslais – analitikas.</t>
         </is>
       </c>
     </row>

</xml_diff>